<commit_message>
Add FISC bank-code lookup button, 16-digit account format, fix duplicated bank suffix
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AiRhVonLy4fKMkDqRzRHkz
</commit_message>
<xml_diff>
--- a/sbom/SBOM.xlsx
+++ b/sbom/SBOM.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SBOM'!$A$1:$N$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SBOM'!$A$1:$N$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:N36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -626,7 +626,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>476b63943eae06d1e29d2287fdd0c8d48fddb4eb27af7c315522ae789b23f8fa</t>
+          <t>8780517d5db50d4e699ff2191ccff1e340975cb282ab9098f4661408a59cde16</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr"/>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>離線啟動檔 start-windows.bat／server.ps1／start-mac-linux.command</t>
+          <t>財金公司 金融機構代號查詢（外部連結）</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1536,17 +1536,17 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>application</t>
+          <t>service</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>專案自有</t>
+          <t>政府/公營事業網站</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>chaifeng666</t>
+          <t>財金資訊股份有限公司</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1556,12 +1556,12 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>repo offline/</t>
+          <t>www.fisc.com.tw（只有按「查銀行代號」時開新分頁）</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>離線版本機伺服器（只接受 localhost）</t>
+          <t>查詢匯款用的 7 碼金融機構代號</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>使用系統內建 Windows PowerShell（Microsoft）或 python3（PSF）</t>
+          <t>只開啟查詢頁，不帶任何資料；分行名稱複製到使用者剪貼簿由使用者自行貼上。總行 3 碼對照表內建在 index.html。</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr"/>
@@ -1583,17 +1583,17 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>ocr-app（本地 OCR 小程式 ocr.html／OCR-offline.zip）</t>
+          <t>ocr-classify-ui（單據分類，GitHub Pages／離線版）</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>ocr.html（自行開發）</t>
+          <t>離線啟動檔 start-windows.bat／server.ps1／start-mac-linux.command</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1618,12 +1618,12 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>/mnt/project-files/ocr-app/</t>
+          <t>repo offline/</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>主程式</t>
+          <t>離線版本機伺服器（只接受 localhost）</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -1631,12 +1631,12 @@
           <t>✅ 通過</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>e8525a839fb0f594135a6000fb34b1a093b898cd379cd5349fe2d6b99439aacd</t>
-        </is>
-      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>使用系統內建 Windows PowerShell（Microsoft）或 python3（PSF）</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1650,42 +1650,42 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>tesseract.js</t>
+          <t>ocr.html（自行開發）</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>5.1.1</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>library</t>
+          <t>application</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Apache-2.0</t>
+          <t>專案自有</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Project Naptha（Kevin Kwok 等）</t>
+          <t>chaifeng666</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>美國</t>
+          <t>臺灣</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>npm registry → OCR-offline.zip lib/；線上版從 jsDelivr 下載</t>
+          <t>/mnt/project-files/ocr-app/</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>OCR 主程式（瀏覽器端）</t>
+          <t>主程式</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -1696,14 +1696,10 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>a8e29918d098b2b06e1012bdaeffb4aec0445c5d5654709023e0bd1f442a80e8</t>
-        </is>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>pkg:npm/tesseract.js@5.1.1</t>
-        </is>
-      </c>
+          <t>e8525a839fb0f594135a6000fb34b1a093b898cd379cd5349fe2d6b99439aacd</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1716,7 +1712,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>tesseract.js worker</t>
+          <t>tesseract.js</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1736,7 +1732,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Project Naptha</t>
+          <t>Project Naptha（Kevin Kwok 等）</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1746,12 +1742,12 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>npm registry → OCR-offline.zip lib/；線上版從 jsDelivr 下載</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>OCR 背景執行緒</t>
+          <t>OCR 主程式（瀏覽器端）</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
@@ -1762,12 +1758,12 @@
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>aca1229639fc9907d86f96e825955a2b7c5716d17f3bc3acd71f9c7ab66181fc</t>
+          <t>a8e29918d098b2b06e1012bdaeffb4aec0445c5d5654709023e0bd1f442a80e8</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>pkg:npm/tesseract.js@5.1.1#worker</t>
+          <t>pkg:npm/tesseract.js@5.1.1</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1778,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>tesseract.js-core（Tesseract OCR 5＋Leptonica，WebAssembly）</t>
+          <t>tesseract.js worker</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1797,12 +1793,12 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Apache-2.0（Tesseract）／BSD-2-Clause（Leptonica）</t>
+          <t>Apache-2.0</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Tesseract：HP → Google，開源社群維護；Leptonica：Dan Bloomberg</t>
+          <t>Project Naptha</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1817,7 +1813,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>OCR 引擎</t>
+          <t>OCR 背景執行緒</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -1825,19 +1821,15 @@
           <t>✅ 通過</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>一般版與 SIMD 加速版各一</t>
-        </is>
-      </c>
+      <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>ce20eda9533cbed1e6c2b4276fbae1e0adc61b6754b5513084be601787b457cf</t>
+          <t>aca1229639fc9907d86f96e825955a2b7c5716d17f3bc3acd71f9c7ab66181fc</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>pkg:npm/tesseract.js-core@5.1.1</t>
+          <t>pkg:npm/tesseract.js@5.1.1#worker</t>
         </is>
       </c>
     </row>
@@ -1852,27 +1844,27 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Tesseract 語言資料 chi_tra（繁體中文）</t>
+          <t>tesseract.js-core（Tesseract OCR 5＋Leptonica，WebAssembly）</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>4.0.0 best_int</t>
+          <t>5.1.1</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>library</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Apache-2.0</t>
+          <t>Apache-2.0（Tesseract）／BSD-2-Clause（Leptonica）</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Google LLC（tessdata）</t>
+          <t>Tesseract：HP → Google，開源社群維護；Leptonica：Dan Bloomberg</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1882,12 +1874,12 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>tesseract.js 官方語言資料 → lib/lang/</t>
+          <t>同上</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>繁體中文辨識模型</t>
+          <t>OCR 引擎</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
@@ -1895,15 +1887,19 @@
           <t>✅ 通過</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>一般版與 SIMD 加速版各一</t>
+        </is>
+      </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>11fe2610dab05d8a880d02f193ce70203f4c4bbe061b987d5529a2c038a22743</t>
+          <t>ce20eda9533cbed1e6c2b4276fbae1e0adc61b6754b5513084be601787b457cf</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>pkg:generic/tessdata/chi_tra@4.0.0</t>
+          <t>pkg:npm/tesseract.js-core@5.1.1</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1914,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Tesseract 語言資料 eng（英文）</t>
+          <t>Tesseract 語言資料 chi_tra（繁體中文）</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1948,12 +1944,12 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>tesseract.js 官方語言資料 → lib/lang/</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>英文辨識模型</t>
+          <t>繁體中文辨識模型</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -1964,12 +1960,12 @@
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>45b4cb346724ac1774f1c36f42f182b887bcdb28ebe63e6fff90ac41f3fcff91</t>
+          <t>11fe2610dab05d8a880d02f193ce70203f4c4bbe061b987d5529a2c038a22743</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>pkg:generic/tessdata/eng@4.0.0</t>
+          <t>pkg:generic/tessdata/chi_tra@4.0.0</t>
         </is>
       </c>
     </row>
@@ -1984,17 +1980,17 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>PDF.js（pdfjs-dist）</t>
+          <t>Tesseract 語言資料 eng（英文）</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>3.11.174</t>
+          <t>4.0.0 best_int</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>library</t>
+          <t>data</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2004,7 +2000,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Mozilla Foundation</t>
+          <t>Google LLC（tessdata）</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -2014,12 +2010,12 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>npm registry → lib/</t>
+          <t>同上</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>讀取 PDF、轉成影像</t>
+          <t>英文辨識模型</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -2030,12 +2026,12 @@
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>5b5799e6f8c680663207ac5b42ee14eed2a406fa7af48f50c154f0c0b1566946</t>
+          <t>45b4cb346724ac1774f1c36f42f182b887bcdb28ebe63e6fff90ac41f3fcff91</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>pkg:npm/pdfjs-dist@3.11.174</t>
+          <t>pkg:generic/tessdata/eng@4.0.0</t>
         </is>
       </c>
     </row>
@@ -2050,7 +2046,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>PDF.js worker</t>
+          <t>PDF.js（pdfjs-dist）</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -2080,12 +2076,12 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>npm registry → lib/</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>PDF 背景解析</t>
+          <t>讀取 PDF、轉成影像</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
@@ -2096,12 +2092,12 @@
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>feabdf309770ed24bba31a5467836cdc8cf639c705af27d52b585b041bb8527b</t>
+          <t>5b5799e6f8c680663207ac5b42ee14eed2a406fa7af48f50c154f0c0b1566946</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>pkg:npm/pdfjs-dist@3.11.174#worker</t>
+          <t>pkg:npm/pdfjs-dist@3.11.174</t>
         </is>
       </c>
     </row>
@@ -2116,27 +2112,27 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Adobe CMap 字元對照表（pdfjs-dist/cmaps）</t>
+          <t>PDF.js worker</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>3.11.174 隨附</t>
+          <t>3.11.174</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>library</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>BSD-3-Clause</t>
+          <t>Apache-2.0</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Adobe Inc.</t>
+          <t>Mozilla Foundation</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -2146,12 +2142,12 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>同上 → lib/cmaps/</t>
+          <t>同上</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>正確讀出 PDF 內的中日韓文字</t>
+          <t>PDF 背景解析</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -2159,13 +2155,17 @@
           <t>✅ 通過</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>檔名有 GB、UniGB 的是「簡體字編碼」的對照表，由 Adobe 製作，不是中國大陸來源的元件；只用來讀取用該編碼存的 PDF。</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>feabdf309770ed24bba31a5467836cdc8cf639c705af27d52b585b041bb8527b</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>pkg:npm/pdfjs-dist@3.11.174#worker</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -2178,27 +2178,27 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>SheetJS（xlsx）</t>
+          <t>Adobe CMap 字元對照表（pdfjs-dist/cmaps）</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>0.18.5</t>
+          <t>3.11.174 隨附</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>library</t>
+          <t>data</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Apache-2.0</t>
+          <t>BSD-3-Clause</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>SheetJS LLC</t>
+          <t>Adobe Inc.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2208,12 +2208,12 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>npm registry → lib/</t>
+          <t>同上 → lib/cmaps/</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>讀寫 Excel</t>
+          <t>正確讀出 PDF 內的中日韓文字</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
@@ -2221,17 +2221,13 @@
           <t>✅ 通過</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr">
-        <is>
-          <t>c9506197caf809a075b6dee1da0d36fb19da7158ffe8a88e7b0c96c5d8623c99</t>
-        </is>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t>pkg:npm/xlsx@0.18.5</t>
-        </is>
-      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>檔名有 GB、UniGB 的是「簡體字編碼」的對照表，由 Adobe 製作，不是中國大陸來源的元件；只用來讀取用該編碼存的 PDF。</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -2244,12 +2240,12 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>mammoth</t>
+          <t>SheetJS（xlsx）</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>1.8.0</t>
+          <t>0.18.5</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2259,17 +2255,17 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>BSD-2-Clause</t>
+          <t>Apache-2.0</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Michael Williamson</t>
+          <t>SheetJS LLC</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>英國</t>
+          <t>美國</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2279,7 +2275,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>讀取 Word（.docx）文字</t>
+          <t>讀寫 Excel</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
@@ -2290,12 +2286,12 @@
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>deb07bf230d1cb3e190bc5adc6743f35c6531b6571d1e5469b24f452a7f0f4ab</t>
+          <t>c9506197caf809a075b6dee1da0d36fb19da7158ffe8a88e7b0c96c5d8623c99</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>pkg:npm/mammoth@1.8.0</t>
+          <t>pkg:npm/xlsx@0.18.5</t>
         </is>
       </c>
     </row>
@@ -2310,12 +2306,12 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>JSZip</t>
+          <t>mammoth</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>3.10.1</t>
+          <t>1.8.0</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2325,12 +2321,12 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>MIT OR GPL-3.0-or-later</t>
+          <t>BSD-2-Clause</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Stuart Knightley</t>
+          <t>Michael Williamson</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2345,7 +2341,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>讀取 PPT、Word 壓縮內容</t>
+          <t>讀取 Word（.docx）文字</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
@@ -2356,12 +2352,12 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>acc7e41455a80765b5fd9c7ee1b8078a6d160bbbca455aeae854de65c947d59e</t>
+          <t>deb07bf230d1cb3e190bc5adc6743f35c6531b6571d1e5469b24f452a7f0f4ab</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>pkg:npm/jszip@3.10.1</t>
+          <t>pkg:npm/mammoth@1.8.0</t>
         </is>
       </c>
     </row>
@@ -2376,42 +2372,42 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>手寫數字辨識模型 DIGIT_NET（自行訓練）</t>
+          <t>JSZip</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>3.10.1</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>library</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>專案自有（訓練資料 CC BY-SA 3.0）</t>
+          <t>MIT OR GPL-3.0-or-later</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>chaifeng666；訓練資料 MNIST（LeCun、Cortes、Burges，源自美國 NIST）</t>
+          <t>Stuart Knightley</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>臺灣（模型）／美國（資料）</t>
+          <t>英國</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>內嵌於 ocr.html</t>
+          <t>npm registry → lib/</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>領據的身分證、電話等數字欄</t>
+          <t>讀取 PPT、Word 壓縮內容</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
@@ -2419,13 +2415,17 @@
           <t>✅ 通過</t>
         </is>
       </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>int8 權重直接寫在 ocr.html 裡，不需下載</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="inlineStr"/>
-      <c r="N30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>acc7e41455a80765b5fd9c7ee1b8078a6d160bbbca455aeae854de65c947d59e</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>pkg:npm/jszip@3.10.1</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2438,42 +2438,42 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>jsDelivr CDN</t>
+          <t>手寫數字辨識模型 DIGIT_NET（自行訓練）</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>service</t>
+          <t>data</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>jsDelivr 服務條款</t>
+          <t>專案自有（訓練資料 CC BY-SA 3.0）</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>jsDelivr（Prospect One，波蘭）；節點由 Cloudflare、Fastly（美國）提供</t>
+          <t>chaifeng666；訓練資料 MNIST（LeCun、Cortes、Burges，源自美國 NIST）</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>波蘭／美國</t>
+          <t>臺灣（模型）／美國（資料）</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>cdn.jsdelivr.net（只有線上載入模式；OCR-offline.zip 不使用）</t>
+          <t>內嵌於 ocr.html</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>下載程式庫與語言資料（只下載，不上傳）</t>
+          <t>領據的身分證、電話等數字欄</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>網頁的安全限制（CSP）只允許連到 jsDelivr 與本機。</t>
+          <t>int8 權重直接寫在 ocr.html 裡，不需下載</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr"/>
@@ -2500,52 +2500,52 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>系統字型：Microsoft JhengHei／PingFang TC／Noto Sans TC</t>
+          <t>jsDelivr CDN</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>系統內建</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>font</t>
+          <t>service</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>系統授權</t>
+          <t>jsDelivr 服務條款</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Microsoft／Apple／Google</t>
+          <t>jsDelivr（Prospect One，波蘭）；節點由 Cloudflare、Fastly（美國）提供</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>美國（發行者）</t>
+          <t>波蘭／美國</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>不隨附、不下載（只寫在字型清單裡）</t>
+          <t>cdn.jsdelivr.net（只有線上載入模式；OCR-offline.zip 不使用）</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>畫面字型</t>
-        </is>
-      </c>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ 需注意</t>
+          <t>下載程式庫與語言資料（只下載，不上傳）</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>✅ 通過</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>PingFang TC 與 Noto Sans TC 依公開資料由「常州華文」（中國大陸）參與中文字形設計；建議從字型清單移除，只留微軟正黑體。</t>
+          <t>網頁的安全限制（CSP）只允許連到 jsDelivr 與本機。</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr"/>
@@ -2562,55 +2562,55 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>離線啟動檔 start-windows.bat／server.ps1／start-mac-linux.command</t>
+          <t>系統字型：Microsoft JhengHei／PingFang TC／Noto Sans TC</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>系統內建</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>application</t>
+          <t>font</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>專案自有</t>
+          <t>系統授權</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>chaifeng666</t>
+          <t>Microsoft／Apple／Google</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>臺灣</t>
+          <t>美國（發行者）</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>OCR-offline.zip</t>
+          <t>不隨附、不下載（只寫在字型清單裡）</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>本機伺服器（只接受 localhost）</t>
-        </is>
-      </c>
-      <c r="K33" s="3" t="inlineStr">
-        <is>
-          <t>✅ 通過</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr"/>
-      <c r="M33" s="2" t="inlineStr">
-        <is>
-          <t>aad96a5f3c721d5f2cef0538091841842d6ae1bc48c8d6089707cb040ba2a6de</t>
-        </is>
-      </c>
+          <t>畫面字型</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ 需注意</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>PingFang TC 與 Noto Sans TC 依公開資料由「常州華文」（中國大陸）參與中文字形設計；建議從字型清單移除，只留微軟正黑體。</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr"/>
       <c r="N33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>PaddleOCR PP-OCRv5</t>
+          <t>離線啟動檔 start-windows.bat／server.ps1／start-mac-linux.command</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2634,45 +2634,45 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>library</t>
+          <t>application</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Apache-2.0</t>
+          <t>專案自有</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>百度（Baidu）</t>
+          <t>chaifeng666</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>中國大陸</t>
+          <t>臺灣</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>已於 2026-10-13 移除</t>
+          <t>OCR-offline.zip</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>（舊版 OCR 引擎）</t>
-        </is>
-      </c>
-      <c r="K34" s="5" t="inlineStr">
-        <is>
-          <t>🗑️ 已移除</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>依使用者規定移除，改用 Tesseract（Google）。目前程式中已無任何引用。</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="inlineStr"/>
+          <t>本機伺服器（只接受 localhost）</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>✅ 通過</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>aad96a5f3c721d5f2cef0538091841842d6ae1bc48c8d6089707cb040ba2a6de</t>
+        </is>
+      </c>
       <c r="N34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
@@ -2686,7 +2686,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>OpenCC</t>
+          <t>PaddleOCR PP-OCRv5</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>BYVoid</t>
+          <t>百度（Baidu）</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>（舊版簡繁轉換）</t>
+          <t>（舊版 OCR 引擎）</t>
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr">
@@ -2731,14 +2731,76 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>依使用者規定移除。目前程式中已無任何引用。</t>
+          <t>依使用者規定移除，改用 Tesseract（Google）。目前程式中已無任何引用。</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="2" t="inlineStr"/>
     </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>ocr-app（本地 OCR 小程式 ocr.html／OCR-offline.zip）</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>OpenCC</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>library</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>BYVoid</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>中國大陸</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>已於 2026-10-13 移除</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>（舊版簡繁轉換）</t>
+        </is>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>🗑️ 已移除</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>依使用者規定移除。目前程式中已無任何引用。</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N35"/>
+  <autoFilter ref="A1:N36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2771,7 +2833,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-25T00:03:39+00:00</t>
+          <t>2026-10-25T00:27:19+00:00</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2856,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Point bank-code lookup to CBC 全國金融機構一覽
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AiRhVonLy4fKMkDqRzRHkz
</commit_message>
<xml_diff>
--- a/sbom/SBOM.xlsx
+++ b/sbom/SBOM.xlsx
@@ -626,7 +626,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>8780517d5db50d4e699ff2191ccff1e340975cb282ab9098f4661408a59cde16</t>
+          <t>6da7662317b22b04fd566f8752a596e1e9be593912d6587e58732cff8d202bb4</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr"/>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>財金公司 金融機構代號查詢（外部連結）</t>
+          <t>中央銀行 全國金融機構一覽查詢（外部連結）</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1541,12 +1541,12 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>政府/公營事業網站</t>
+          <t>政府網站</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>財金資訊股份有限公司</t>
+          <t>中央銀行</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>www.fisc.com.tw（只有按「查銀行代號」時開新分頁）</t>
+          <t>www.cbc.gov.tw（只有按「查銀行代號」時開新分頁）</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -2833,7 +2833,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-25T00:27:19+00:00</t>
+          <t>2026-10-25T00:35:36+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>